<commit_message>
docs: revise workplan Phase 4 to the one-scale-robust-model plan
Rewrote the Phase 4 task rows (32-42) in edmonds_combined_workplan.xlsx from the old
per-year/per-tier fine-tune to the unified plan (cozy-skipping-jellyfish.md): Phase A
foundation, B deciduous SEMANTIC hand-labels, C one scale-robust RGB train, D honest
C-CAP/NDVI eval + Olofsson harness, E apply-all + validate, F reconcile docs. Gate 2
now requires independent (C-CAP + Olofsson) validation, not the circular number.
Row count + Gantt fills + all other phases preserved. Backup in _archive.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scripts/edmonds_combined_workplan.xlsx
+++ b/Scripts/edmonds_combined_workplan.xlsx
@@ -952,7 +952,7 @@
     <row r="32">
       <c r="A32" s="40" t="inlineStr">
         <is>
-          <t>PHASE 4: PER-YEAR FINE-TUNING — SEMANTIC SEGMENTATION (17 YEARS) (IN PROGRESS)</t>
+          <t>PHASE 4: ONE SCALE-ROBUST SEMANTIC MODEL — LABELS-FIRST (REVISED 2026-07-10; plan=cozy-skipping-jellyfish.md; 18 years, native resolution)</t>
         </is>
       </c>
       <c r="B32" s="36" t="n"/>
@@ -973,7 +973,7 @@
     <row r="33" ht="23" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Temporal-anchor label transfer: approve/reject 2020 crowns vs each year at control years (2000/2020/2024); assign validity intervals</t>
+          <t>Phase A Foundation (mostly done): Forest_4 spectral check (2016 NDVI 0.61 ~= conifer, NOT the missed variety); honest-metric bugs fixed; quarantine broken 2022/2017 runs</t>
         </is>
       </c>
       <c r="D33" s="36" t="n"/>
@@ -982,7 +982,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Region-based labels: mark non-canopy background (lawn, roof, road, water) to fix negative scarcity; review scales with temporal distance</t>
+          <t>Phase B Hand-trace SEMANTIC canopy extent at the missed low-NDVI deciduous stands (forest_miss_stands_2016/2015) at 2016 (coarse, NIR-verifiable) + a fine year; C-CAP locates only; keep an eval split</t>
         </is>
       </c>
       <c r="D34" s="36" t="n"/>
@@ -991,7 +991,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Per-tier fine-tune (fine/medium/coarse) from the 2020 anchor + LiDAR canopy-height (CHM) 4th channel to reject grass false-positives; single scale-robust model deferred</t>
+          <t>Phase C Train ONE scale-robust RGB model: pooled multi-resolution labels + strong multi-scale/downscale augmentation, v039 recipe, two-phase from the 2020 anchor (replaces per-tier fine-tune)</t>
         </is>
       </c>
       <c r="E35" s="36" t="n"/>
@@ -1000,7 +1000,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Full-city native-resolution inference → per-year canopy probability raster + binary mask</t>
+          <t>Phase D Honest evaluation: independent C-CAP + NDVI+CHM (report bracketed); target forest recall ~0.80+ with precision held. CHM/NDVI inform LABELS only, never a model input</t>
         </is>
       </c>
       <c r="F36" s="36" t="n"/>
@@ -1009,7 +1009,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Resample all per-year masks to a common coarse grid for apples-to-apples temporal comparison</t>
+          <t>Phase D Build the Olofsson (2014) stratified photo-interp harness (area-adjusted accuracy + 95% CIs) — deliverable-grade arbiter, essential for pre-2016 years with no independent reference</t>
         </is>
       </c>
       <c r="G37" s="36" t="n"/>
@@ -1018,7 +1018,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Threshold-independent evaluation: AUROC, average precision, best-F1 operating point per year</t>
+          <t>Phase E Apply the one model to all 18 acquisitions at native resolution -&gt; per-year canopy probability + mask rasters (no upscaling)</t>
         </is>
       </c>
       <c r="F38" s="36" t="n"/>
@@ -1028,7 +1028,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Independent validation: NDVI+CHM reference for the 4 NIR years (honest recall) + random-point i-Tree photo-interpretation for all years incl. no-NIR 2000</t>
+          <t>Phase E Validate: no fine-vs-coarse recall cliff at a common threshold; cross-year canopy-area consistency + non-tree-parcel flicker</t>
         </is>
       </c>
       <c r="F39" s="36" t="n"/>
@@ -1039,7 +1039,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Concentrate human review on oldest/coarse years (2000, 2002) + mixed-residential + negatives — NOTE: the 14,476-crown 2020 review is not yet complete</t>
+          <t>Phase F Reconcile Method_Pipeline.md + pipeline_buildtracker.md to the unified method; retire the cross-sensor experiment to validation-later</t>
         </is>
       </c>
       <c r="F40" s="36" t="n"/>
@@ -1050,7 +1050,7 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>◆ DECISION GATE 2: Do per-year semantic masks pass random-point photo-interpretation (i-Tree)? Include / exclude / flag low-confidence (esp. coarse 2000/2002)</t>
+          <t>DECISION GATE 2: Do the per-year semantic masks pass INDEPENDENT validation — C-CAP + Olofsson random-point photo-interp — at target recall/precision (NOT the circular 2020-mask number)?</t>
         </is>
       </c>
       <c r="F42" s="37" t="n"/>

</xml_diff>